<commit_message>
Updated  module and fixed UI issues
</commit_message>
<xml_diff>
--- a/out_custom.xlsx
+++ b/out_custom.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>SNo</t>
   </si>
@@ -26,7 +26,7 @@
     <t>PIS</t>
   </si>
   <si>
-    <t>ACCNO</t>
+    <t>BANK_ACCNO</t>
   </si>
   <si>
     <t>GPFPRAN</t>
@@ -41,6 +41,9 @@
     <t>2008AE10</t>
   </si>
   <si>
+    <t>10000000001</t>
+  </si>
+  <si>
     <t>GPF-1111</t>
   </si>
   <si>
@@ -51,6 +54,9 @@
   </si>
   <si>
     <t>2008AE12</t>
+  </si>
+  <si>
+    <t>10000000010</t>
   </si>
   <si>
     <t>GPF-2222</t>
@@ -139,7 +145,7 @@
         <v>9</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -147,19 +153,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>